<commit_message>
Enhanced prompt and Retrieval optimizations
</commit_message>
<xml_diff>
--- a/Retrieval_accuracy_test.xlsx
+++ b/Retrieval_accuracy_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mnemosyne\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2891188C-361A-42D9-81F0-9D17EB01AD47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EE62DB-3770-40F6-AAC2-37346465CE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98712C83-EEA3-4AF6-BFB0-AD51C6A96C9B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="62">
   <si>
     <t>#</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Question</t>
   </si>
   <si>
-    <t>Retrieved Video(s)</t>
-  </si>
-  <si>
     <t>Expected Video(s)</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>10, 12</t>
   </si>
   <si>
-    <t>10,12</t>
-  </si>
-  <si>
     <t>actually good</t>
   </si>
   <si>
@@ -184,6 +178,48 @@
   </si>
   <si>
     <t>suggest to refer video 17. also recommended to check another resource that specifically covers graph algorithms and data structures</t>
+  </si>
+  <si>
+    <t>Optimized RAG Retirved</t>
+  </si>
+  <si>
+    <t>Original Retrieved Video(s)</t>
+  </si>
+  <si>
+    <t>4, 11, 10</t>
+  </si>
+  <si>
+    <t>4 or 5, 10</t>
+  </si>
+  <si>
+    <t>13, 14, 15</t>
+  </si>
+  <si>
+    <t>17, 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5, 7 </t>
+  </si>
+  <si>
+    <t>Optimized RAG Quality</t>
+  </si>
+  <si>
+    <t>Unfortunately, the requested topic "JavaScript DOM manipulation" is not explicitly mentioned in this video. However, the instructor briefly mentions HTML, CSS, and JavaScript, which might be related to DOM manipulation in a broader sense.</t>
+  </si>
+  <si>
+    <t>13, 11, 14</t>
+  </si>
+  <si>
+    <t>may be right even expected is something else</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5, 4 </t>
+  </si>
+  <si>
+    <t>In this video, the instructor mentions React, but only briefly. They say "there is a little problem. Then I will tell you React, then you will say, what is happening? Then," but they don't explain or demonstrate React itself. That is its forcing answers.</t>
+  </si>
+  <si>
+    <t>I couldn't find this topic in the course material.</t>
   </si>
 </sst>
 </file>
@@ -227,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -238,10 +274,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -558,19 +591,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9371A18-A648-4350-8A50-6BCE05A625E3}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="3"/>
     <col min="2" max="2" width="98.109375" style="2" customWidth="1"/>
     <col min="3" max="3" width="22.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="3"/>
-    <col min="7" max="7" width="20" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" style="3" customWidth="1"/>
+    <col min="5" max="6" width="25.88671875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="27.88671875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="53.44140625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -578,27 +613,33 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3">
         <v>0.70573667502604798</v>
@@ -609,16 +650,19 @@
       <c r="E2" s="3">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G2" s="3">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C3" s="3">
         <v>0.69962027647281499</v>
@@ -629,16 +673,19 @@
       <c r="E3" s="3">
         <v>5</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G3" s="3">
+        <v>5</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3">
         <v>0.68267305304570902</v>
@@ -649,16 +696,19 @@
       <c r="E4" s="3">
         <v>7</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="3">
         <v>0.72235018139212204</v>
@@ -669,16 +719,19 @@
       <c r="E5" s="3">
         <v>8</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G5" s="3">
+        <v>8</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="3">
         <v>0.68120495681714499</v>
@@ -689,16 +742,19 @@
       <c r="E6" s="3">
         <v>9</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G6" s="3">
+        <v>9</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>12</v>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="C7" s="3">
         <v>0.67059250524809999</v>
@@ -709,16 +765,19 @@
       <c r="E7" s="3">
         <v>11</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G7" s="3">
+        <v>11</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="3">
         <v>0.69053469921180499</v>
@@ -729,16 +788,19 @@
       <c r="E8" s="3">
         <v>10</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G8" s="3">
+        <v>10</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="3">
         <v>0.64791075314731705</v>
@@ -746,19 +808,25 @@
       <c r="D9" s="3">
         <v>1</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="E9" s="3">
+        <v>7</v>
+      </c>
+      <c r="G9" s="3">
+        <v>7</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I9" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="3">
         <v>0.69473979140333397</v>
@@ -769,19 +837,22 @@
       <c r="E10" s="3">
         <v>8</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G10" s="3">
+        <v>8</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3">
         <v>0.70379961395613</v>
@@ -792,16 +863,19 @@
       <c r="E11" s="3">
         <v>17</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G11" s="3">
+        <v>17</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>17</v>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C12" s="3">
         <v>0.67731552514010396</v>
@@ -810,18 +884,21 @@
         <v>18</v>
       </c>
       <c r="E12" s="3">
+        <v>13</v>
+      </c>
+      <c r="G12" s="3">
         <v>18</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>36</v>
+      <c r="B13" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="C13" s="3">
         <v>0.64353542232716099</v>
@@ -832,19 +909,22 @@
       <c r="E13" s="3">
         <v>6</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G13" s="3">
+        <v>6</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" s="3">
         <v>0.71350250639382595</v>
@@ -852,42 +932,48 @@
       <c r="D14" s="3">
         <v>5</v>
       </c>
-      <c r="E14" s="3">
-        <v>5</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="3">
         <v>0.73078875776299401</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="3">
+        <v>12</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="3">
         <v>0.70287483928848704</v>
@@ -898,19 +984,22 @@
       <c r="E16" s="3">
         <v>14</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G16" s="3">
+        <v>14</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3">
         <v>0.62378560085660795</v>
@@ -921,16 +1010,19 @@
       <c r="E17" s="3">
         <v>17</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G17" s="3">
+        <v>17</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="3">
         <v>0.68916691883730796</v>
@@ -941,99 +1033,120 @@
       <c r="E18" s="3">
         <v>11</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G18" s="3">
+        <v>11</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="3">
         <v>0.69265379975191099</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="3">
         <v>0.66897253955937896</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C21" s="3">
         <v>0.67981106914974099</v>
       </c>
       <c r="D21" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22" s="3">
         <v>0.59087821544681096</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" s="3">
         <v>0.647981456103221</v>
@@ -1042,18 +1155,21 @@
         <v>4</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C24" s="3">
         <v>0.57126568957157497</v>
@@ -1062,38 +1178,50 @@
         <v>4</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C25" s="3">
         <v>0.52941291017722603</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" s="3">
         <v>0.50221578922848298</v>
@@ -1102,21 +1230,27 @@
         <v>17</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C27" s="3">
         <v>0.47669799083856501</v>
@@ -1125,10 +1259,16 @@
         <v>1</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>34</v>
+        <v>61</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>